<commit_message>
Update Live Traffic [Sat Jul 18 04:17:53 UTC 2026]
</commit_message>
<xml_diff>
--- a/datos/live_today.xlsx
+++ b/datos/live_today.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH1"/>
+  <dimension ref="A1:AH14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -597,6 +601,1805 @@
       <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Delay</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>23001091</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Pacific Telecom Group S.A.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>447728705510</v>
+      </c>
+      <c r="F2" t="n">
+        <v>234</v>
+      </c>
+      <c r="G2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Hutchison 3G UK Ltd</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>ASMSC_OK</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>T2W_SIM</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Yahoo</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="Q2" s="2" t="n">
+        <v>46221.01092592593</v>
+      </c>
+      <c r="R2" s="2" t="n">
+        <v>46221.01096064815</v>
+      </c>
+      <c r="S2" s="2" t="n">
+        <v>46221.01100694444</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="V2" t="n">
+        <v>1</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>UCS2</t>
+        </is>
+      </c>
+      <c r="X2" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dbab0c82-98f9-4a28-9bd9-5d117f7bec7f              </t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bc864c45-7735-47cf-9779-f22a571e9aed              </t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>Hi there. 074 295</t>
+        </is>
+      </c>
+      <c r="AG2" t="n">
+        <v>7</v>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>7 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>23001090</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Pacific Telecom Group S.A.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>447403281197</v>
+      </c>
+      <c r="F3" t="n">
+        <v>234</v>
+      </c>
+      <c r="G3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Hutchison 3G UK Ltd</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>ASMSC_OK</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>T2W_SIM</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Yahoo</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>46221.0106712963</v>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>46221.01069444444</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>46221.01086805556</v>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
+        <v>1</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="X3" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AC3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9849eda3-7e09-4715-b9eb-aff724ff2b31              </t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6c6fadf9-c783-40e8-831e-a014c3e49ff4              </t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>Hi there. 664 567</t>
+        </is>
+      </c>
+      <c r="AG3" t="n">
+        <v>17</v>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>17 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>23001089</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Pacific Telecom Group S.A.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>447590822820</v>
+      </c>
+      <c r="F4" t="n">
+        <v>234</v>
+      </c>
+      <c r="G4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Telefonica UK Limited</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>ASMSC_OK</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>T2W_SIM</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Yahoo</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>46221.00864583333</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>46221.00866898148</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>46221.00881944445</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>1</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="X4" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ed18aff8-eff0-4add-8653-9f92e3213293              </t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8398c128-4ee0-4bea-816a-f1d2024ca662              </t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Hi there. 763 457</t>
+        </is>
+      </c>
+      <c r="AG4" t="n">
+        <v>15</v>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>15 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>23001088</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Pacific Telecom Group S.A.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>447986136180</v>
+      </c>
+      <c r="F5" t="n">
+        <v>234</v>
+      </c>
+      <c r="G5" t="n">
+        <v>30</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>EE Limited ( TM)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>ASMSC_OK</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>T2W_SIM</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Yahoo</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>46221.00633101852</v>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>46221.00636574074</v>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>46221.00659722222</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="V5" t="n">
+        <v>1</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="X5" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AC5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d6ddb17e-6083-4cc2-a8f7-82ab5c1e2e6d              </t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3e258f7e-096f-46ae-b5dd-808f7151290d              </t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>Hi there. 869 380</t>
+        </is>
+      </c>
+      <c r="AG5" t="n">
+        <v>23</v>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>23 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>23001087</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Pacific Telecom Group S.A.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PTG_DIR</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>PSG_DIR</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>5581995012721</v>
+      </c>
+      <c r="F6" t="n">
+        <v>724</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>CUBIC TELECOM BRASIL LTDA</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>ASMSC_OK</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>KPERU_HQ</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>CLICKSMS</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>46221.00585648148</v>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>46221.00587962963</v>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>46221.00604166667</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="V6" t="n">
+        <v>1</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="X6" t="n">
+        <v>56</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>-1</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0.0047</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0.0047</v>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AC6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">daa07ad4-6c43-4cb8-acaa-5f9e72cecdda              </t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cd2c173c-a12f-01f2-b75e-9c6b003e96d8              </t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CAT TROVA..
+-3.82729,-32.40796
+CAT TROVA?O EM MOVIMENTO
+</t>
+        </is>
+      </c>
+      <c r="AG6" t="n">
+        <v>16</v>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>16 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>23001086</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Pacific Telecom Group S.A.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>447440173543</v>
+      </c>
+      <c r="F7" t="n">
+        <v>234</v>
+      </c>
+      <c r="G7" t="n">
+        <v>26</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Lycamobile UK Limited</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>ASMSC_OK</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>T2W_SIM</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Yahoo</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>46221.00559027777</v>
+      </c>
+      <c r="R7" s="2" t="n">
+        <v>46221.005625</v>
+      </c>
+      <c r="S7" s="2" t="n">
+        <v>46221.0056712963</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>1</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="X7" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">780808ec-07a7-410a-91a7-6a1b30a89c80              </t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">db0ac408-446b-4d06-aef5-66fecf63088c              </t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>Hi there. 638 922</t>
+        </is>
+      </c>
+      <c r="AG7" t="n">
+        <v>7</v>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>7 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>23001085</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Pacific Telecom Group S.A.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>447913405159</v>
+      </c>
+      <c r="F8" t="n">
+        <v>234</v>
+      </c>
+      <c r="G8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>EE Limited ( TM)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>ASMSC_OK</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>T2W_SIM</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Yahoo</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="Q8" s="2" t="n">
+        <v>46221.00538194444</v>
+      </c>
+      <c r="R8" s="2" t="n">
+        <v>46221.00539351852</v>
+      </c>
+      <c r="S8" s="2" t="n">
+        <v>46221.00552083334</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="V8" t="n">
+        <v>1</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="X8" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y8" t="inlineStr"/>
+      <c r="Z8" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AC8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6855840e-6cf9-4923-b6b9-37a6a2c34af0              </t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c1da2efd-9d83-4905-8d91-8077c87f0f96              </t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>Hi there. 370 547</t>
+        </is>
+      </c>
+      <c r="AG8" t="n">
+        <v>12</v>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>12 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>23001084</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Pacific Telecom Group S.A.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>447478315678</v>
+      </c>
+      <c r="F9" t="n">
+        <v>234</v>
+      </c>
+      <c r="G9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Hutchison 3G UK Ltd</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>ASMSC_OK</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>T2W_SIM</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Yahoo</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="Q9" s="2" t="n">
+        <v>46221.00450231481</v>
+      </c>
+      <c r="R9" s="2" t="n">
+        <v>46221.00452546297</v>
+      </c>
+      <c r="S9" s="2" t="n">
+        <v>46221.00467592593</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="V9" t="n">
+        <v>1</v>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="X9" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AC9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">de3fa669-363b-4e22-9e30-356eb6f75f3d              </t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8b1126d9-dcf2-49b7-8382-f4fcb4322d3b              </t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>Hi there. 051 438</t>
+        </is>
+      </c>
+      <c r="AG9" t="n">
+        <v>15</v>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>15 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>23001083</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Pacific Telecom Group S.A.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>447988321760</v>
+      </c>
+      <c r="F10" t="n">
+        <v>234</v>
+      </c>
+      <c r="G10" t="n">
+        <v>20</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Hutchison 3G UK Ltd</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>ASMSC_OK</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>T2W_SIM</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Yahoo</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="Q10" s="2" t="n">
+        <v>46221.00431712963</v>
+      </c>
+      <c r="R10" s="2" t="n">
+        <v>46221.00434027778</v>
+      </c>
+      <c r="S10" s="2" t="n">
+        <v>46221.00440972222</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="V10" t="n">
+        <v>1</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>UCS2</t>
+        </is>
+      </c>
+      <c r="X10" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AC10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1cba22d2-fb23-4c77-af5b-9bd4bbeeb05c              </t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">648b4f8a-28ae-4fe0-b584-930e7d869225              </t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>Hi there. 292 049</t>
+        </is>
+      </c>
+      <c r="AG10" t="n">
+        <v>8</v>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>8 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>23001082</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Pacific Telecom Group S.A.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>447956172818</v>
+      </c>
+      <c r="F11" t="n">
+        <v>234</v>
+      </c>
+      <c r="G11" t="n">
+        <v>30</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>EE Limited ( TM)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>ASMSC_OK</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>T2W_SIM</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Yahoo</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>46221.003125</v>
+      </c>
+      <c r="R11" s="2" t="n">
+        <v>46221.00314814815</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>46221.0033912037</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="V11" t="n">
+        <v>1</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="X11" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AC11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3985f8fa-2ec2-465c-be6f-9e2d335c1beb              </t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7a367272-d93f-4b23-b36a-abfef7e030e5              </t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>Hi there. 300 356</t>
+        </is>
+      </c>
+      <c r="AG11" t="n">
+        <v>23</v>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>23 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>23001081</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Pacific Telecom Group S.A.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>447446828323</v>
+      </c>
+      <c r="F12" t="n">
+        <v>234</v>
+      </c>
+      <c r="G12" t="n">
+        <v>20</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Hutchison 3G UK Ltd</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>ASMSC_OK</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>T2W_SIM</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Yahoo</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>46221.00293981482</v>
+      </c>
+      <c r="R12" s="2" t="n">
+        <v>46221.00296296296</v>
+      </c>
+      <c r="S12" s="2" t="n">
+        <v>46221.00305555556</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="V12" t="n">
+        <v>1</v>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="X12" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AC12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ab537c34-a64e-4662-b110-7004f807eece              </t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">afa673d7-fae4-4de8-8bb9-7321fa31192a              </t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>Hi there. 299 841</t>
+        </is>
+      </c>
+      <c r="AG12" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>10 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>23001080</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Pacific Telecom Group S.A.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>447590822820</v>
+      </c>
+      <c r="F13" t="n">
+        <v>234</v>
+      </c>
+      <c r="G13" t="n">
+        <v>10</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Telefonica UK Limited</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>ASMSC_OK</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>T2W_SIM</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Yahoo</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>46221.00239583333</v>
+      </c>
+      <c r="R13" s="2" t="n">
+        <v>46221.00241898148</v>
+      </c>
+      <c r="S13" s="2" t="n">
+        <v>46221.00261574074</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="V13" t="n">
+        <v>1</v>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="X13" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y13" t="inlineStr"/>
+      <c r="Z13" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AC13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a889d3f5-f2e6-43ed-8335-32db6f05805f              </t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0e4df1de-335c-4ae4-8b6f-e3965d35031b              </t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>Hi there. 215 187</t>
+        </is>
+      </c>
+      <c r="AG13" t="n">
+        <v>19</v>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>19 seconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>23001079</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pacific Telecom Group S.A.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>PTG_SIM</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>447830348495</v>
+      </c>
+      <c r="F14" t="n">
+        <v>234</v>
+      </c>
+      <c r="G14" t="n">
+        <v>20</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Hutchison 3G UK Ltd</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>ASMSC_OK</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>T2W_SIM</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Yahoo</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>46221.00021990741</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>46221.00025462963</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>46221.00030092592</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>SMPP</t>
+        </is>
+      </c>
+      <c r="V14" t="n">
+        <v>1</v>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Default</t>
+        </is>
+      </c>
+      <c r="X14" t="n">
+        <v>17</v>
+      </c>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AA14" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="AC14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">536e3488-79ab-44d2-92d6-360153b1368f              </t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6c261771-d245-4fdd-a10e-2f746cdeecdf              </t>
+        </is>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>Hi there. 876 857</t>
+        </is>
+      </c>
+      <c r="AG14" t="n">
+        <v>7</v>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>7 seconds</t>
         </is>
       </c>
     </row>

</xml_diff>